<commit_message>
Add payment receive and KPI metadata support
</commit_message>
<xml_diff>
--- a/excel_import/business_data_import_template.xlsx
+++ b/excel_import/business_data_import_template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="12500" yWindow="600" windowWidth="25820" windowHeight="19260" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4420" yWindow="1200" windowWidth="25820" windowHeight="19260" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
@@ -14,7 +14,7 @@
     <sheet name="Sotephwar_Inventory" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -864,7 +864,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="12" t="n">
@@ -911,7 +910,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="12" t="n">
@@ -958,7 +956,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="12" t="n">
@@ -1005,7 +1002,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6" ht="26" customHeight="1">
       <c r="A6" s="12" t="n">
@@ -1052,7 +1048,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="12" t="n">
@@ -1099,7 +1094,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="12" t="n">
@@ -1146,7 +1140,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="12" t="n">
@@ -1193,7 +1186,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="12" t="n">
@@ -1240,7 +1232,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="12" t="n">
@@ -1287,7 +1278,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="12" t="n">
@@ -1334,7 +1324,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="12" t="n">
@@ -1381,7 +1370,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14" ht="26" customHeight="1">
       <c r="A14" s="12" t="n">
@@ -1428,7 +1416,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="12" t="n">
@@ -1475,7 +1462,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="12" t="n">
@@ -1522,7 +1508,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="12" t="n">
@@ -1569,7 +1554,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18" ht="26" customHeight="1">
       <c r="A18" s="12" t="n">
@@ -1616,7 +1600,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="12" t="n">
@@ -1663,7 +1646,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20" ht="26" customHeight="1">
       <c r="A20" s="12" t="n">
@@ -1710,7 +1692,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21" ht="26" customHeight="1">
       <c r="A21" s="12" t="n">
@@ -1757,7 +1738,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22" ht="26" customHeight="1">
       <c r="A22" s="12" t="n">
@@ -1804,7 +1784,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23" ht="26" customHeight="1">
       <c r="A23" s="12" t="n">
@@ -1851,7 +1830,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24" ht="26" customHeight="1">
       <c r="A24" s="12" t="n">
@@ -1898,7 +1876,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25" ht="26" customHeight="1">
       <c r="A25" s="12" t="n">
@@ -1945,7 +1922,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26" ht="26" customHeight="1">
       <c r="A26" s="12" t="n">
@@ -1992,7 +1968,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27" ht="26" customHeight="1">
       <c r="A27" s="12" t="n">
@@ -2039,7 +2014,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="12" t="n">
@@ -2086,7 +2060,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29" ht="26" customHeight="1">
       <c r="A29" s="12" t="n">
@@ -2133,7 +2106,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30" ht="26" customHeight="1">
       <c r="A30" s="12" t="n">
@@ -2180,7 +2152,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31" ht="26" customHeight="1">
       <c r="A31" s="12" t="n">
@@ -2227,7 +2198,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32" ht="26" customHeight="1">
       <c r="A32" s="12" t="n">
@@ -2274,7 +2244,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33" ht="26" customHeight="1">
       <c r="A33" s="12" t="n">
@@ -2321,7 +2290,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34" ht="26" customHeight="1">
       <c r="A34" s="12" t="n">
@@ -2368,7 +2336,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35" ht="26" customHeight="1">
       <c r="A35" s="12" t="n">
@@ -2415,7 +2382,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36" ht="26" customHeight="1">
       <c r="A36" s="12" t="n">
@@ -2462,7 +2428,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37" ht="26" customHeight="1">
       <c r="A37" s="12" t="n">
@@ -2509,7 +2474,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38" ht="26" customHeight="1">
       <c r="A38" s="12" t="n">
@@ -2556,7 +2520,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39" ht="26" customHeight="1">
       <c r="A39" s="12" t="n">
@@ -2603,7 +2566,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40" ht="26" customHeight="1">
       <c r="A40" s="12" t="n">
@@ -2650,7 +2612,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41" ht="26" customHeight="1">
       <c r="A41" s="12" t="n">
@@ -2697,7 +2658,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42" ht="26" customHeight="1">
       <c r="A42" s="12" t="n">
@@ -2744,7 +2704,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43" ht="26" customHeight="1">
       <c r="A43" s="12" t="n">
@@ -2791,7 +2750,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44" ht="26" customHeight="1">
       <c r="A44" s="12" t="n">
@@ -2838,7 +2796,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45" ht="26" customHeight="1">
       <c r="A45" s="12" t="n">
@@ -2885,7 +2842,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr"/>
     </row>
     <row r="46" ht="26" customHeight="1">
       <c r="A46" s="12" t="n">
@@ -2932,7 +2888,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47" ht="26" customHeight="1">
       <c r="A47" s="12" t="n">
@@ -2979,7 +2934,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48" ht="26" customHeight="1">
       <c r="A48" s="12" t="n">
@@ -3026,7 +2980,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49" ht="26" customHeight="1">
       <c r="A49" s="12" t="n">
@@ -3071,7 +3024,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50" ht="26" customHeight="1">
       <c r="A50" s="12" t="n">
@@ -3118,7 +3070,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51" ht="26" customHeight="1">
       <c r="A51" s="12" t="n">
@@ -3165,7 +3116,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52" ht="26" customHeight="1">
       <c r="A52" s="12" t="n">
@@ -3212,7 +3162,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53" ht="26" customHeight="1">
       <c r="A53" s="12" t="n">
@@ -3259,7 +3208,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54" ht="26" customHeight="1">
       <c r="A54" s="12" t="n">
@@ -3306,7 +3254,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55" ht="26" customHeight="1">
       <c r="A55" s="12" t="n">
@@ -3353,7 +3300,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr"/>
     </row>
     <row r="56" ht="26" customHeight="1">
       <c r="A56" s="12" t="n">
@@ -3400,7 +3346,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr"/>
     </row>
     <row r="57" ht="26" customHeight="1">
       <c r="A57" s="12" t="n">
@@ -3447,7 +3392,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr"/>
     </row>
     <row r="58" ht="26" customHeight="1">
       <c r="A58" s="12" t="n">
@@ -3494,7 +3438,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr"/>
     </row>
     <row r="59" ht="26" customHeight="1">
       <c r="A59" s="12" t="n">
@@ -3541,7 +3484,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr"/>
     </row>
     <row r="60" ht="26" customHeight="1">
       <c r="A60" s="12" t="n">
@@ -3588,7 +3530,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr"/>
     </row>
     <row r="61" ht="26" customHeight="1">
       <c r="A61" s="12" t="n">
@@ -3635,7 +3576,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr"/>
     </row>
     <row r="62" ht="26" customHeight="1">
       <c r="A62" s="12" t="n">
@@ -3682,7 +3622,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M62" t="inlineStr"/>
     </row>
     <row r="63" ht="26" customHeight="1">
       <c r="A63" s="12" t="n">
@@ -3729,7 +3668,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M63" t="inlineStr"/>
     </row>
     <row r="64" ht="26" customHeight="1">
       <c r="A64" s="12" t="n">
@@ -3776,7 +3714,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M64" t="inlineStr"/>
     </row>
     <row r="65" ht="26" customHeight="1">
       <c r="A65" s="12" t="n">
@@ -3823,7 +3760,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M65" t="inlineStr"/>
     </row>
     <row r="66" ht="26" customHeight="1">
       <c r="A66" s="12" t="n">
@@ -3870,7 +3806,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M66" t="inlineStr"/>
     </row>
     <row r="67" ht="26" customHeight="1">
       <c r="A67" s="12" t="n">
@@ -3917,7 +3852,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M67" t="inlineStr"/>
     </row>
     <row r="68" ht="26" customHeight="1">
       <c r="A68" s="12" t="n">
@@ -3964,7 +3898,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M68" t="inlineStr"/>
     </row>
     <row r="69" ht="26" customHeight="1">
       <c r="A69" s="12" t="n">
@@ -4011,7 +3944,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M69" t="inlineStr"/>
     </row>
     <row r="70" ht="26" customHeight="1">
       <c r="A70" s="12" t="n">
@@ -4058,7 +3990,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M70" t="inlineStr"/>
     </row>
     <row r="71" ht="26" customHeight="1">
       <c r="A71" s="12" t="n">
@@ -4105,7 +4036,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M71" t="inlineStr"/>
     </row>
     <row r="72" ht="26" customHeight="1">
       <c r="A72" s="12" t="n">
@@ -4152,7 +4082,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M72" t="inlineStr"/>
     </row>
     <row r="73" ht="26" customHeight="1">
       <c r="A73" s="12" t="n">
@@ -4199,7 +4128,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M73" t="inlineStr"/>
     </row>
     <row r="74" ht="26" customHeight="1">
       <c r="A74" s="12" t="n">
@@ -4246,7 +4174,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M74" t="inlineStr"/>
     </row>
     <row r="75" ht="26" customHeight="1">
       <c r="A75" s="12" t="n">
@@ -4293,7 +4220,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M75" t="inlineStr"/>
     </row>
     <row r="76" ht="26" customHeight="1">
       <c r="A76" s="12" t="n">
@@ -4340,7 +4266,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M76" t="inlineStr"/>
     </row>
     <row r="77" ht="26" customHeight="1">
       <c r="A77" s="12" t="n">
@@ -4387,7 +4312,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M77" t="inlineStr"/>
     </row>
     <row r="78" ht="26" customHeight="1">
       <c r="A78" s="12" t="n">
@@ -4434,7 +4358,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M78" t="inlineStr"/>
     </row>
     <row r="79" ht="26" customHeight="1">
       <c r="A79" s="12" t="n">
@@ -4481,7 +4404,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M79" t="inlineStr"/>
     </row>
     <row r="80" ht="26" customHeight="1">
       <c r="A80" s="12" t="n">
@@ -4528,7 +4450,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M80" t="inlineStr"/>
     </row>
     <row r="81" ht="26" customHeight="1">
       <c r="A81" s="12" t="n">
@@ -4575,7 +4496,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M81" t="inlineStr"/>
     </row>
     <row r="82" ht="26" customHeight="1">
       <c r="A82" s="12" t="n">
@@ -4622,7 +4542,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M82" t="inlineStr"/>
     </row>
     <row r="83" ht="26" customHeight="1">
       <c r="A83" s="12" t="n">
@@ -4669,7 +4588,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M83" t="inlineStr"/>
     </row>
     <row r="84" ht="26" customHeight="1">
       <c r="A84" s="12" t="n">
@@ -4716,7 +4634,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M84" t="inlineStr"/>
     </row>
     <row r="85" ht="26" customHeight="1">
       <c r="A85" s="12" t="n">
@@ -4763,7 +4680,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M85" t="inlineStr"/>
     </row>
     <row r="86" ht="26" customHeight="1">
       <c r="A86" s="12" t="n">
@@ -4810,7 +4726,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M86" t="inlineStr"/>
     </row>
     <row r="87" ht="26" customHeight="1">
       <c r="A87" s="12" t="n">
@@ -4857,7 +4772,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M87" t="inlineStr"/>
     </row>
     <row r="88" ht="26" customHeight="1">
       <c r="A88" s="12" t="n">
@@ -4904,7 +4818,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M88" t="inlineStr"/>
     </row>
     <row r="89" ht="26" customHeight="1">
       <c r="A89" s="12" t="n">
@@ -4951,7 +4864,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M89" t="inlineStr"/>
     </row>
     <row r="90" ht="26" customHeight="1">
       <c r="A90" s="12" t="n">
@@ -4998,7 +4910,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M90" t="inlineStr"/>
     </row>
     <row r="91" ht="26" customHeight="1">
       <c r="A91" s="12" t="n">
@@ -5045,7 +4956,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M91" t="inlineStr"/>
     </row>
     <row r="92" ht="26" customHeight="1">
       <c r="A92" s="12" t="n">
@@ -5092,7 +5002,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M92" t="inlineStr"/>
     </row>
     <row r="93" ht="26" customHeight="1">
       <c r="A93" s="12" t="n">
@@ -5139,7 +5048,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M93" t="inlineStr"/>
     </row>
     <row r="94" ht="26" customHeight="1">
       <c r="A94" s="12" t="n">
@@ -5186,7 +5094,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M94" t="inlineStr"/>
     </row>
     <row r="95" ht="26" customHeight="1">
       <c r="A95" s="12" t="n">
@@ -5233,7 +5140,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M95" t="inlineStr"/>
     </row>
     <row r="96" ht="26" customHeight="1">
       <c r="A96" s="12" t="n">
@@ -5280,7 +5186,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M96" t="inlineStr"/>
     </row>
     <row r="97" ht="26" customHeight="1">
       <c r="A97" s="12" t="n">
@@ -5327,7 +5232,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M97" t="inlineStr"/>
     </row>
     <row r="98" ht="26" customHeight="1">
       <c r="A98" s="12" t="n">
@@ -5374,7 +5278,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M98" t="inlineStr"/>
     </row>
     <row r="99" ht="26" customHeight="1">
       <c r="A99" s="12" t="n">
@@ -5421,7 +5324,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M99" t="inlineStr"/>
     </row>
     <row r="100" ht="26" customHeight="1">
       <c r="A100" s="12" t="n">
@@ -5468,7 +5370,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="12" t="n">
@@ -5515,7 +5416,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M101" t="inlineStr"/>
     </row>
     <row r="102" ht="26" customHeight="1">
       <c r="A102" s="12" t="n">
@@ -5562,7 +5462,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M102" t="inlineStr"/>
     </row>
     <row r="103" ht="26" customHeight="1">
       <c r="A103" s="12" t="n">
@@ -5609,7 +5508,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M103" t="inlineStr"/>
     </row>
     <row r="104" ht="26" customHeight="1">
       <c r="A104" s="12" t="n">
@@ -5656,7 +5554,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M104" t="inlineStr"/>
     </row>
     <row r="105" ht="26" customHeight="1">
       <c r="A105" s="12" t="n">
@@ -5703,7 +5600,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M105" t="inlineStr"/>
     </row>
     <row r="106" ht="26" customHeight="1">
       <c r="A106" s="12" t="n">
@@ -5750,7 +5646,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M106" t="inlineStr"/>
     </row>
     <row r="107" ht="26" customHeight="1">
       <c r="A107" s="12" t="n">
@@ -5797,7 +5692,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M107" t="inlineStr"/>
     </row>
     <row r="108" ht="26" customHeight="1">
       <c r="A108" s="12" t="n">
@@ -5844,7 +5738,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M108" t="inlineStr"/>
     </row>
     <row r="109" ht="26" customHeight="1">
       <c r="A109" s="12" t="n">
@@ -5891,7 +5784,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M109" t="inlineStr"/>
     </row>
     <row r="110" ht="26" customHeight="1">
       <c r="A110" s="12" t="n">
@@ -5938,7 +5830,6 @@
           <t>2026-06-15 21:40:03</t>
         </is>
       </c>
-      <c r="M110" t="inlineStr"/>
     </row>
     <row r="111" ht="26" customHeight="1">
       <c r="A111" s="16" t="n"/>
@@ -12750,256 +12641,1788 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="n"/>
-      <c r="D47" s="9" t="n"/>
-      <c r="E47" s="9" t="n"/>
+      <c r="A47" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>200</v>
+      </c>
+      <c r="D47" s="9" t="n">
+        <v>6600000</v>
+      </c>
+      <c r="E47" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F47" s="9" t="n"/>
+      <c r="H47" s="5" t="n">
+        <v>46187</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Kaung Kyaw</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L47" t="n">
+        <v>685</v>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="n"/>
-      <c r="D48" s="9" t="n"/>
-      <c r="E48" s="9" t="n"/>
+      <c r="A48" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Sote Phwar 4L</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>20</v>
+      </c>
+      <c r="D48" s="9" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="E48" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F48" s="9" t="n"/>
+      <c r="H48" s="5" t="n">
+        <v>46187</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Kaung Kyaw</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L48" t="n">
+        <v>686</v>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="n"/>
-      <c r="D49" s="9" t="n"/>
-      <c r="E49" s="9" t="n"/>
+      <c r="A49" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Sote Phwar 4L</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>4</v>
+      </c>
+      <c r="D49" s="9" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E49" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F49" s="9" t="n"/>
+      <c r="H49" s="5" t="n">
+        <v>46187</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Khin Mar Lwin,Daw</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L49" t="n">
+        <v>687</v>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="n"/>
-      <c r="D50" s="9" t="n"/>
-      <c r="E50" s="9" t="n"/>
+      <c r="A50" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>200</v>
+      </c>
+      <c r="D50" s="9" t="n">
+        <v>6600000</v>
+      </c>
+      <c r="E50" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F50" s="9" t="n"/>
+      <c r="H50" s="5" t="n">
+        <v>46187</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Zun Ei Khaing</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L50" t="n">
+        <v>688</v>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="n"/>
-      <c r="D51" s="9" t="n"/>
-      <c r="E51" s="9" t="n"/>
+      <c r="A51" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Sote Phwar 4L</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>8</v>
+      </c>
+      <c r="D51" s="9" t="n">
+        <v>960000</v>
+      </c>
+      <c r="E51" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F51" s="9" t="n"/>
+      <c r="H51" s="5" t="n">
+        <v>46187</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Zun Ei Khaing</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L51" t="n">
+        <v>689</v>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="n"/>
-      <c r="D52" s="9" t="n"/>
-      <c r="E52" s="9" t="n"/>
+      <c r="A52" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>210</v>
+      </c>
+      <c r="D52" s="9" t="n">
+        <v>6600000</v>
+      </c>
+      <c r="E52" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F52" s="9" t="n"/>
+      <c r="H52" s="5" t="n">
+        <v>46187</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Laye Yar Myay</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L52" t="n">
+        <v>690</v>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="n"/>
-      <c r="D53" s="9" t="n"/>
-      <c r="E53" s="9" t="n"/>
+      <c r="A53" s="6" t="n">
+        <v>56</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>10</v>
+      </c>
+      <c r="D53" s="9" t="n">
+        <v>330000</v>
+      </c>
+      <c r="E53" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F53" s="9" t="n"/>
+      <c r="H53" s="5" t="n">
+        <v>46187</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>ZLP</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L53" t="n">
+        <v>691</v>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="n"/>
-      <c r="D54" s="9" t="n"/>
-      <c r="E54" s="9" t="n"/>
+      <c r="A54" s="6" t="n">
+        <v>56</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Sote Phwar 500 mL</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>20</v>
+      </c>
+      <c r="D54" s="9" t="n">
+        <v>340000</v>
+      </c>
+      <c r="E54" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F54" s="9" t="n"/>
+      <c r="H54" s="5" t="n">
+        <v>46187</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>ZLP</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L54" t="n">
+        <v>692</v>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="6" t="n"/>
-      <c r="D55" s="9" t="n"/>
-      <c r="E55" s="9" t="n"/>
-      <c r="F55" s="9" t="n"/>
+      <c r="A55" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>1100</v>
+      </c>
+      <c r="D55" s="9" t="n">
+        <v>32500000</v>
+      </c>
+      <c r="E55" s="9" t="n">
+        <v>32500000</v>
+      </c>
+      <c r="F55" s="9" t="inlineStr">
+        <is>
+          <t>14.6.2026 Paid MM&amp;17.6.2026 Paid MM</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="n">
+        <v>46188</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Lucky 7</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L55" t="n">
+        <v>693</v>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="6" t="n"/>
-      <c r="D56" s="9" t="n"/>
-      <c r="E56" s="9" t="n"/>
-      <c r="F56" s="9" t="n"/>
+      <c r="A56" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Sote Phwar 500 mL</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>300</v>
+      </c>
+      <c r="D56" s="9" t="n">
+        <v>5100000</v>
+      </c>
+      <c r="E56" s="9" t="n">
+        <v>5100000</v>
+      </c>
+      <c r="F56" s="9" t="inlineStr">
+        <is>
+          <t>14.6.2026 Paid MM</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="n">
+        <v>46188</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Lucky 7</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L56" t="n">
+        <v>694</v>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="6" t="n"/>
-      <c r="D57" s="9" t="n"/>
-      <c r="E57" s="9" t="n"/>
-      <c r="F57" s="9" t="n"/>
+      <c r="A57" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>1100</v>
+      </c>
+      <c r="D57" s="9" t="n">
+        <v>32500000</v>
+      </c>
+      <c r="E57" s="9" t="n">
+        <v>32500000</v>
+      </c>
+      <c r="F57" s="9" t="inlineStr">
+        <is>
+          <t>17.6.2026 Paid MM</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="n">
+        <v>46188</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Mya Yadanar</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L57" t="n">
+        <v>695</v>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="n"/>
-      <c r="D58" s="9" t="n"/>
-      <c r="E58" s="9" t="n"/>
-      <c r="F58" s="9" t="n"/>
+      <c r="A58" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Sote Phwar 500 mL</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>400</v>
+      </c>
+      <c r="D58" s="9" t="n">
+        <v>6800000</v>
+      </c>
+      <c r="E58" s="9" t="n">
+        <v>6800000</v>
+      </c>
+      <c r="F58" s="9" t="inlineStr">
+        <is>
+          <t>17.6.2026 Paid MM</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="n">
+        <v>46188</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Mya Yadanar</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L58" t="n">
+        <v>696</v>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="n"/>
-      <c r="D59" s="9" t="n"/>
-      <c r="E59" s="9" t="n"/>
+      <c r="A59" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Sote Phwar 4L</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>4</v>
+      </c>
+      <c r="D59" s="9" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E59" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F59" s="9" t="n"/>
+      <c r="H59" s="5" t="n">
+        <v>46188</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Aye Su</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L59" t="n">
+        <v>697</v>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="n"/>
-      <c r="D60" s="9" t="n"/>
-      <c r="E60" s="9" t="n"/>
+      <c r="A60" s="6" t="n">
+        <v>61</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D60" s="9" t="n">
+        <v>33000000</v>
+      </c>
+      <c r="E60" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F60" s="9" t="n"/>
+      <c r="H60" s="5" t="n">
+        <v>46189</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Ko Aung Aung</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L60" t="n">
+        <v>698</v>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="6" t="n"/>
-      <c r="D61" s="9" t="n"/>
-      <c r="E61" s="9" t="n"/>
+      <c r="A61" s="6" t="n">
+        <v>61</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Sote Phwar 500 mL</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D61" s="9" t="n">
+        <v>34000000</v>
+      </c>
+      <c r="E61" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F61" s="9" t="n"/>
+      <c r="H61" s="5" t="n">
+        <v>46189</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Ko Aung Aung</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L61" t="n">
+        <v>699</v>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="6" t="n"/>
-      <c r="D62" s="9" t="n"/>
-      <c r="E62" s="9" t="n"/>
+      <c r="A62" s="6" t="n">
+        <v>62</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Sote Phwar 500 mL</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>100</v>
+      </c>
+      <c r="D62" s="9" t="n">
+        <v>1700000</v>
+      </c>
+      <c r="E62" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F62" s="9" t="n"/>
+      <c r="H62" s="5" t="n">
+        <v>46189</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Aungthapyay</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L62" t="n">
+        <v>700</v>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="6" t="n"/>
-      <c r="D63" s="9" t="n"/>
-      <c r="E63" s="9" t="n"/>
+      <c r="A63" s="6" t="n">
+        <v>63</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>500</v>
+      </c>
+      <c r="D63" s="9" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="E63" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F63" s="9" t="n"/>
+      <c r="H63" s="5" t="n">
+        <v>46189</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Pwint Aung Kyaw POL</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L63" t="n">
+        <v>701</v>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="6" t="n"/>
-      <c r="D64" s="9" t="n"/>
-      <c r="E64" s="9" t="n"/>
+      <c r="A64" s="6" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Sote Phwar 500 mL</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>200</v>
+      </c>
+      <c r="D64" s="9" t="n">
+        <v>3400000</v>
+      </c>
+      <c r="E64" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F64" s="9" t="n"/>
+      <c r="H64" s="5" t="n">
+        <v>46189</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Pwint Aung Kyaw POL</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L64" t="n">
+        <v>702</v>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="6" t="n"/>
-      <c r="D65" s="9" t="n"/>
-      <c r="E65" s="9" t="n"/>
+      <c r="A65" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>1100</v>
+      </c>
+      <c r="D65" s="9" t="n">
+        <v>33000000</v>
+      </c>
+      <c r="E65" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F65" s="9" t="n"/>
+      <c r="H65" s="5" t="n">
+        <v>46189</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Shwe War</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L65" t="n">
+        <v>703</v>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="6" t="n"/>
-      <c r="D66" s="9" t="n"/>
-      <c r="E66" s="9" t="n"/>
+      <c r="A66" s="6" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>100</v>
+      </c>
+      <c r="D66" s="9" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="E66" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F66" s="9" t="n"/>
+      <c r="H66" s="5" t="n">
+        <v>46189</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Moe Myint Min(PW)</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L66" t="n">
+        <v>704</v>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="6" t="n"/>
-      <c r="D67" s="9" t="n"/>
-      <c r="E67" s="9" t="n"/>
+      <c r="A67" s="6" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Sote Phwar 500 mL</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>20</v>
+      </c>
+      <c r="D67" s="9" t="n">
+        <v>340000</v>
+      </c>
+      <c r="E67" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F67" s="9" t="n"/>
+      <c r="H67" s="5" t="n">
+        <v>46189</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Moe Myint Min(PW)</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L67" t="n">
+        <v>705</v>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="6" t="n"/>
-      <c r="D68" s="9" t="n"/>
-      <c r="E68" s="9" t="n"/>
+      <c r="A68" s="6" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>210</v>
+      </c>
+      <c r="D68" s="9" t="n">
+        <v>6600000</v>
+      </c>
+      <c r="E68" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F68" s="9" t="n"/>
+      <c r="H68" s="5" t="n">
+        <v>46189</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Aung Kyaw Swe</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L68" t="n">
+        <v>706</v>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="6" t="n"/>
-      <c r="D69" s="9" t="n"/>
-      <c r="E69" s="9" t="n"/>
+      <c r="A69" s="6" t="n">
+        <v>66</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Sote Phwar 4L</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>4</v>
+      </c>
+      <c r="D69" s="9" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E69" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F69" s="9" t="n"/>
+      <c r="H69" s="5" t="n">
+        <v>46189</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Aung Kyaw Swe</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L69" t="n">
+        <v>707</v>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="6" t="n"/>
-      <c r="D70" s="9" t="n"/>
-      <c r="E70" s="9" t="n"/>
+      <c r="A70" s="6" t="n">
+        <v>67</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>50</v>
+      </c>
+      <c r="D70" s="9" t="n">
+        <v>1650000</v>
+      </c>
+      <c r="E70" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F70" s="9" t="n"/>
+      <c r="H70" s="5" t="n">
+        <v>46189</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Phyo Thein Kywal</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L70" t="n">
+        <v>708</v>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="6" t="n"/>
-      <c r="D71" s="9" t="n"/>
-      <c r="E71" s="9" t="n"/>
+      <c r="A71" s="6" t="n">
+        <v>68</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>100</v>
+      </c>
+      <c r="D71" s="9" t="n">
+        <v>3300000</v>
+      </c>
+      <c r="E71" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F71" s="9" t="n"/>
+      <c r="H71" s="5" t="n">
+        <v>46189</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Da Na Phyo Kywal</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L71" t="n">
+        <v>709</v>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="6" t="n"/>
-      <c r="D72" s="9" t="n"/>
-      <c r="E72" s="9" t="n"/>
+      <c r="A72" s="6" t="n">
+        <v>69</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>150</v>
+      </c>
+      <c r="D72" s="9" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="E72" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F72" s="9" t="n"/>
+      <c r="H72" s="5" t="n">
+        <v>46189</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Pwint Aung Kyaw</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L72" t="n">
+        <v>710</v>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="6" t="n"/>
-      <c r="D73" s="9" t="n"/>
-      <c r="E73" s="9" t="n"/>
+      <c r="A73" s="6" t="n">
+        <v>69</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Sote Phwar 4L</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>8</v>
+      </c>
+      <c r="D73" s="9" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E73" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F73" s="9" t="n"/>
+      <c r="H73" s="5" t="n">
+        <v>46189</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Pwint Aung Kyaw</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L73" t="n">
+        <v>711</v>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="6" t="n"/>
-      <c r="D74" s="9" t="n"/>
-      <c r="E74" s="9" t="n"/>
+      <c r="A74" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D74" s="9" t="n">
+        <v>33000000</v>
+      </c>
+      <c r="E74" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F74" s="9" t="n"/>
+      <c r="H74" s="5" t="n">
+        <v>46190</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Myat Nyi Aung</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L74" t="n">
+        <v>712</v>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="6" t="n"/>
-      <c r="D75" s="9" t="n"/>
-      <c r="E75" s="9" t="n"/>
+      <c r="A75" s="6" t="n">
+        <v>71</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>40</v>
+      </c>
+      <c r="D75" s="9" t="n">
+        <v>1320000</v>
+      </c>
+      <c r="E75" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F75" s="9" t="n"/>
+      <c r="H75" s="5" t="n">
+        <v>46190</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Ya Way Chit Oo</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L75" t="n">
+        <v>713</v>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="6" t="n"/>
-      <c r="D76" s="9" t="n"/>
-      <c r="E76" s="9" t="n"/>
+      <c r="A76" s="6" t="n">
+        <v>71</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Sote Phwar 500 mL</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>20</v>
+      </c>
+      <c r="D76" s="9" t="n">
+        <v>340000</v>
+      </c>
+      <c r="E76" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F76" s="9" t="n"/>
+      <c r="H76" s="5" t="n">
+        <v>46190</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Ya Way Chit Oo</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L76" t="n">
+        <v>714</v>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="6" t="n"/>
-      <c r="D77" s="9" t="n"/>
-      <c r="E77" s="9" t="n"/>
+      <c r="A77" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>210</v>
+      </c>
+      <c r="D77" s="9" t="n">
+        <v>6600000</v>
+      </c>
+      <c r="E77" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F77" s="9" t="n"/>
+      <c r="H77" s="5" t="n">
+        <v>46190</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Aung Kyaw Hein</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L77" t="n">
+        <v>715</v>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="6" t="n"/>
-      <c r="D78" s="9" t="n"/>
-      <c r="E78" s="9" t="n"/>
+      <c r="A78" s="6" t="n">
+        <v>73</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Sote Phwar 500 mL</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>100</v>
+      </c>
+      <c r="D78" s="9" t="n">
+        <v>1700000</v>
+      </c>
+      <c r="E78" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F78" s="9" t="n"/>
+      <c r="H78" s="5" t="n">
+        <v>46190</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Theint Theint Thu</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L78" t="n">
+        <v>716</v>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="6" t="n"/>
-      <c r="D79" s="9" t="n"/>
-      <c r="E79" s="9" t="n"/>
+      <c r="A79" s="6" t="n">
+        <v>74</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>30</v>
+      </c>
+      <c r="D79" s="9" t="n">
+        <v>990000</v>
+      </c>
+      <c r="E79" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F79" s="9" t="n"/>
+      <c r="H79" s="5" t="n">
+        <v>46190</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Hein Zaw Phyo</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L79" t="n">
+        <v>717</v>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="6" t="n"/>
-      <c r="D80" s="9" t="n"/>
-      <c r="E80" s="9" t="n"/>
+      <c r="A80" s="6" t="n">
+        <v>75</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>30</v>
+      </c>
+      <c r="D80" s="9" t="n">
+        <v>990000</v>
+      </c>
+      <c r="E80" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F80" s="9" t="n"/>
+      <c r="H80" s="5" t="n">
+        <v>46190</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Da Na Phyo Kywal</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L80" t="n">
+        <v>718</v>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="6" t="n"/>
-      <c r="D81" s="9" t="n"/>
-      <c r="E81" s="9" t="n"/>
+      <c r="A81" s="6" t="n">
+        <v>76</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>10</v>
+      </c>
+      <c r="D81" s="9" t="n">
+        <v>330000</v>
+      </c>
+      <c r="E81" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F81" s="9" t="n"/>
+      <c r="H81" s="5" t="n">
+        <v>46190</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Hein Zaw Phyo</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L81" t="n">
+        <v>719</v>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="6" t="n"/>
-      <c r="D82" s="9" t="n"/>
-      <c r="E82" s="9" t="n"/>
+      <c r="A82" s="6" t="n">
+        <v>76</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Sote Phwar 4L</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>4</v>
+      </c>
+      <c r="D82" s="9" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E82" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F82" s="9" t="n"/>
+      <c r="H82" s="5" t="n">
+        <v>46190</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Hein Zaw Phyo</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L82" t="n">
+        <v>720</v>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="6" t="n"/>
-      <c r="D83" s="9" t="n"/>
-      <c r="E83" s="9" t="n"/>
-      <c r="F83" s="9" t="n"/>
+      <c r="A83" s="6" t="n">
+        <v>77</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>105</v>
+      </c>
+      <c r="D83" s="9" t="n">
+        <v>3300000</v>
+      </c>
+      <c r="E83" s="9" t="n">
+        <v>3300000</v>
+      </c>
+      <c r="F83" s="9" t="inlineStr">
+        <is>
+          <t>18.6.2026 Paid Kpay MM</t>
+        </is>
+      </c>
+      <c r="H83" s="5" t="n">
+        <v>46191</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Thee Pwint San</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L83" t="n">
+        <v>721</v>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="6" t="n"/>
-      <c r="D84" s="9" t="n"/>
-      <c r="E84" s="9" t="n"/>
+      <c r="A84" s="6" t="n">
+        <v>78</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>110</v>
+      </c>
+      <c r="D84" s="9" t="n">
+        <v>3135000</v>
+      </c>
+      <c r="E84" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F84" s="9" t="n"/>
+      <c r="H84" s="5" t="n">
+        <v>46191</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Zun Ei Khaing</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L84" t="n">
+        <v>722</v>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" s="6" t="n"/>
-      <c r="D85" s="9" t="n"/>
-      <c r="E85" s="9" t="n"/>
+      <c r="A85" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>100</v>
+      </c>
+      <c r="D85" s="9" t="n">
+        <v>3300000</v>
+      </c>
+      <c r="E85" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F85" s="9" t="n"/>
+      <c r="H85" s="5" t="n">
+        <v>46191</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Billion</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L85" t="n">
+        <v>723</v>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="6" t="n"/>
-      <c r="D86" s="9" t="n"/>
-      <c r="E86" s="9" t="n"/>
+      <c r="A86" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>210</v>
+      </c>
+      <c r="D86" s="9" t="n">
+        <v>6600000</v>
+      </c>
+      <c r="E86" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F86" s="9" t="n"/>
+      <c r="H86" s="5" t="n">
+        <v>46192</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Kaung Kin Pyar</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L86" t="n">
+        <v>724</v>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="6" t="n"/>
-      <c r="D87" s="9" t="n"/>
-      <c r="E87" s="9" t="n"/>
+      <c r="A87" s="6" t="n">
+        <v>81</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Sote Phwar 500 mL</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>100</v>
+      </c>
+      <c r="D87" s="9" t="n">
+        <v>1700000</v>
+      </c>
+      <c r="E87" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F87" s="9" t="n"/>
+      <c r="H87" s="5" t="n">
+        <v>46192</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Cetena</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L87" t="n">
+        <v>725</v>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="6" t="n"/>
-      <c r="D88" s="9" t="n"/>
-      <c r="E88" s="9" t="n"/>
+      <c r="A88" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Sote Phwar 1 L</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>20</v>
+      </c>
+      <c r="D88" s="9" t="n">
+        <v>660000</v>
+      </c>
+      <c r="E88" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F88" s="9" t="n"/>
+      <c r="H88" s="5" t="n">
+        <v>46192</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Myat Bone Saung</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="L88" t="n">
+        <v>726</v>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:24</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="6" t="n"/>

</xml_diff>

<commit_message>
Release Business OS v1.0 - Unified Excel Audit & Import
</commit_message>
<xml_diff>
--- a/excel_import/business_data_import_template.xlsx
+++ b/excel_import/business_data_import_template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19380" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19300" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
@@ -10078,88 +10078,928 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n"/>
+      <c r="A2" s="3" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>77</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2786200</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2786200</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>130</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n"/>
+      <c r="A3" s="3" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>78</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1843100</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1843100</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>131</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n"/>
+      <c r="A4" s="3" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>79</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3375000</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3375000</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>132</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
+      <c r="A5" s="3" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>80</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1990900</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1990900</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>133</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n"/>
+      <c r="A6" s="3" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>81</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3633000</v>
+      </c>
+      <c r="E6" t="n">
+        <v>3633000</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>134</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n"/>
+      <c r="A7" s="3" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>82</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2118200</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2118200</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>135</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n"/>
+      <c r="A8" s="3" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>83</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3108000</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3108000</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>136</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n"/>
+      <c r="A9" s="3" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>84</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1778800</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1778800</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>137</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n"/>
+      <c r="A10" s="3" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>85</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3384500</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3384500</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>138</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n"/>
+      <c r="A11" s="3" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>86</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2087000</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2087000</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>139</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n"/>
+      <c r="A12" s="3" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>87</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3523200</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3523200</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>140</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n"/>
+      <c r="A13" s="3" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>88</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2610500</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2610500</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>141</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n"/>
+      <c r="A14" s="3" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>89</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3747000</v>
+      </c>
+      <c r="E14" t="n">
+        <v>3747000</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>142</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n"/>
+      <c r="A15" s="3" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>90</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2858000</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2858000</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>143</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n"/>
+      <c r="A16" s="3" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>91</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3263000</v>
+      </c>
+      <c r="E16" t="n">
+        <v>3263000</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>144</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n"/>
+      <c r="A17" s="3" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>92</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2707500</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2707500</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>145</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n"/>
+      <c r="A18" s="3" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>93</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2661000</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2661000</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>146</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n"/>
+      <c r="A19" s="3" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>94</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1899900</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1899900</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>147</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n"/>
+      <c r="A20" s="3" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>95</v>
+      </c>
+      <c r="D20" t="n">
+        <v>968000</v>
+      </c>
+      <c r="E20" t="n">
+        <v>968000</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>148</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n"/>
+      <c r="A21" s="3" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>96</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1284000</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1284000</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>149</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n"/>
+      <c r="A22" s="3" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>97</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3414700</v>
+      </c>
+      <c r="E22" t="n">
+        <v>3414700</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>150</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n"/>
+      <c r="A23" s="3" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>98</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1937400</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1937400</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>151</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="n"/>
+      <c r="A24" s="3" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>99</v>
+      </c>
+      <c r="D24" t="n">
+        <v>184000</v>
+      </c>
+      <c r="E24" t="n">
+        <v>184000</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>152</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n"/>
+      <c r="A25" s="3" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>100</v>
+      </c>
+      <c r="D25" t="n">
+        <v>92000</v>
+      </c>
+      <c r="E25" t="n">
+        <v>92000</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>153</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="n"/>
+      <c r="A26" s="3" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>101</v>
+      </c>
+      <c r="D26" t="n">
+        <v>3517500</v>
+      </c>
+      <c r="E26" t="n">
+        <v>3517500</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>154</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="n"/>
+      <c r="A27" s="3" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>102</v>
+      </c>
+      <c r="D27" t="n">
+        <v>2196400</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2196400</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>155</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="n"/>
+      <c r="A28" s="3" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>103</v>
+      </c>
+      <c r="D28" t="n">
+        <v>4703500</v>
+      </c>
+      <c r="E28" t="n">
+        <v>4703500</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>156</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="n"/>
+      <c r="A29" s="3" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Makro</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>104</v>
+      </c>
+      <c r="D29" t="n">
+        <v>2410400</v>
+      </c>
+      <c r="E29" t="n">
+        <v>2410400</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>INSERTED</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>157</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:13:50</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n"/>
@@ -10752,7 +11592,6 @@
           <t>2026-07-21 00:32:05</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -10802,7 +11641,6 @@
           <t>2026-07-21 00:32:05</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">

</xml_diff>